<commit_message>
update to excel builder
</commit_message>
<xml_diff>
--- a/public/ptt.xlsx
+++ b/public/ptt.xlsx
@@ -194,12 +194,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
@@ -208,6 +202,12 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -547,7 +547,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10"/>
@@ -557,11 +557,11 @@
       <c r="F1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="14"/>
+      <c r="H1" s="12"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="10"/>
@@ -571,7 +571,7 @@
       <c r="F2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="15"/>
+      <c r="H2" s="13"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
@@ -586,16 +586,16 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
@@ -652,12 +652,12 @@
         <v>10</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
@@ -678,12 +678,12 @@
         <v>12</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
xuat hang and thu tien
</commit_message>
<xml_diff>
--- a/public/ptt.xlsx
+++ b/public/ptt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diepm\Desktop\git\diepgia-management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D9D2F4-B843-4BD4-9E0C-6D99C65EB60B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD0EEC3-8344-48A3-BCD2-D7233B0689C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>Lý do thu :</t>
   </si>
   <si>
-    <t>Nơi nhận</t>
-  </si>
-  <si>
     <t>Người thu tiền</t>
   </si>
   <si>
@@ -87,6 +84,9 @@
   </si>
   <si>
     <t>Ngày thu :</t>
+  </si>
+  <si>
+    <t>Nơi nhận:</t>
   </si>
 </sst>
 </file>
@@ -97,7 +97,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="[$-1010409]d/m/yyyy\ h:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,13 +142,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -158,7 +151,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -166,11 +159,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -178,40 +186,37 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,37 +547,38 @@
     <col min="2" max="2" width="8.78515625" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="6" max="6" width="9.42578125" customWidth="1"/>
-    <col min="7" max="7" width="14.640625" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="8.640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="G1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="12"/>
-      <c r="I1" s="2"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10" t="s">
-        <v>15</v>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="G2" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="H2" s="13"/>
-      <c r="I2" s="2"/>
+      <c r="I2" s="13"/>
     </row>
     <row r="3" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
@@ -586,117 +592,116 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="22.5" x14ac:dyDescent="0.6">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="16"/>
-      <c r="G5" s="8" t="s">
+      <c r="F5" s="9"/>
+      <c r="G5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="2"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="2"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="2"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="2"/>
+      <c r="A10" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
     </row>
     <row r="11" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2" t="s">
-        <v>14</v>
+      <c r="F11" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -746,11 +751,17 @@
       <c r="I15" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="10">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="C8:I8"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="C10:H10"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="C10:I10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="11" orientation="landscape" r:id="rId1"/>

</xml_diff>